<commit_message>
added references for amphibians
</commit_message>
<xml_diff>
--- a/Project_clone/Report/primer_data.xlsx
+++ b/Project_clone/Report/primer_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
   <si>
     <t xml:space="preserve">Typ av analys</t>
   </si>
@@ -85,6 +85,9 @@
     <t xml:space="preserve">60-55</t>
   </si>
   <si>
+    <t xml:space="preserve">Prie et al. 2021</t>
+  </si>
+  <si>
     <t xml:space="preserve">St. vattensalamander</t>
   </si>
   <si>
@@ -161,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">AAGACGAAAAGACCCCGC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zieritz et al. 2012</t>
   </si>
   <si>
     <t xml:space="preserve">Fisk (16S)</t>
@@ -283,7 +289,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -294,6 +300,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -516,19 +526,22 @@
       <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="G4" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>60</v>
@@ -536,16 +549,16 @@
     </row>
     <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>60</v>
@@ -553,16 +566,16 @@
     </row>
     <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>60</v>
@@ -570,47 +583,47 @@
     </row>
     <row r="8" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>10</v>
@@ -621,7 +634,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>18</v>
@@ -638,13 +651,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>10</v>
@@ -652,62 +665,65 @@
       <c r="E12" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="G12" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="3" t="s">
         <v>49</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>51</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="4" t="s">
         <v>58</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>59</v>
+      <c r="F15" s="4" t="s">
+        <v>61</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>